<commit_message>
Temporarily removed sample data
</commit_message>
<xml_diff>
--- a/notebooks/settings.xlsx
+++ b/notebooks/settings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Documents/_Plato/Plato/notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD70D80-2D4E-A146-9A68-346A7B449842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94524058-4AA8-C848-85DE-458A2FE16C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="2" xr2:uid="{745898CB-6A96-6A42-A7F0-C6C371FC8CE9}"/>
   </bookViews>
@@ -1655,7 +1655,7 @@
         <v>3.0099999999999998E-2</v>
       </c>
       <c r="G8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="4">
         <v>5100000000000</v>

</xml_diff>

<commit_message>
Apparently managed to solve plate tectonics?
</commit_message>
<xml_diff>
--- a/notebooks/settings.xlsx
+++ b/notebooks/settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Documents/_Plato/Plato/notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94524058-4AA8-C848-85DE-458A2FE16C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E40710B-A8B0-F94F-853F-98A27C97090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="2" xr2:uid="{745898CB-6A96-6A42-A7F0-C6C371FC8CE9}"/>
+    <workbookView xWindow="-20760" yWindow="-20460" windowWidth="28800" windowHeight="16280" activeTab="2" xr2:uid="{745898CB-6A96-6A42-A7F0-C6C371FC8CE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Notebook 2 - Optimisation old" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Fixed continental keels and removing net rotation
</commit_message>
<xml_diff>
--- a/notebooks/settings.xlsx
+++ b/notebooks/settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Documents/_Plato/Plato/notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E40710B-A8B0-F94F-853F-98A27C97090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF248FD-C46E-F844-BE31-A9BF204B237E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20760" yWindow="-20460" windowWidth="28800" windowHeight="16280" activeTab="2" xr2:uid="{745898CB-6A96-6A42-A7F0-C6C371FC8CE9}"/>
+    <workbookView xWindow="19620" yWindow="-20880" windowWidth="28800" windowHeight="16280" activeTab="2" xr2:uid="{745898CB-6A96-6A42-A7F0-C6C371FC8CE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Notebook 2 - Optimisation old" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="37">
   <si>
     <t>Name</t>
   </si>
@@ -119,6 +119,36 @@
   </si>
   <si>
     <t>slab suction constant</t>
+  </si>
+  <si>
+    <t>LAB depth threshold</t>
+  </si>
+  <si>
+    <t>Depth-dependent mantle drag</t>
+  </si>
+  <si>
+    <t>ref_NNR</t>
+  </si>
+  <si>
+    <t>seds_NNR</t>
+  </si>
+  <si>
+    <t>keels_NNR</t>
+  </si>
+  <si>
+    <t>suction_NNR</t>
+  </si>
+  <si>
+    <t>seds_keels_NNR</t>
+  </si>
+  <si>
+    <t>seds_suction_NNR</t>
+  </si>
+  <si>
+    <t>keels_suction_NNR</t>
+  </si>
+  <si>
+    <t>seds_keels_suction_NNR</t>
   </si>
 </sst>
 </file>
@@ -1039,17 +1069,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE4CBD66-BFAB-B949-8E50-D28214CEE213}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1063,13 +1095,16 @@
         <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1085,11 +1120,14 @@
       <c r="E2" t="b">
         <v>0</v>
       </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F2" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1105,11 +1143,14 @@
       <c r="E3" t="b">
         <v>0</v>
       </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F3" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1125,111 +1166,129 @@
       <c r="E4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="F4" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E6" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1245,11 +1304,14 @@
       <c r="E10" t="b">
         <v>0</v>
       </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1265,11 +1327,14 @@
       <c r="E11" t="b">
         <v>0</v>
       </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F11" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1285,107 +1350,125 @@
       <c r="E12" t="b">
         <v>1</v>
       </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
+      <c r="F12" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="C13" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="b">
         <v>0</v>
       </c>
-      <c r="C14" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
+      <c r="B15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+      <c r="B16" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="5" t="b">
+      <c r="B17" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4">
+        <v>150000</v>
+      </c>
+      <c r="G17" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1396,22 +1479,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A7984F9-5B2E-0F42-9830-D8CBB6318A94}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1431,19 +1514,22 @@
         <v>19</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1451,7 +1537,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
@@ -1460,22 +1546,25 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
       </c>
       <c r="H2" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I2" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1483,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D3" s="2" t="b">
         <v>1</v>
@@ -1492,22 +1581,25 @@
         <v>1000</v>
       </c>
       <c r="F3" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H3" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I3" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1515,7 +1607,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D4" s="2" t="b">
         <v>0</v>
@@ -1524,22 +1616,25 @@
         <v>0</v>
       </c>
       <c r="F4" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G4" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I4" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1547,7 +1642,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -1555,23 +1650,26 @@
       <c r="E5" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="1">
-        <v>3.0099999999999998E-2</v>
+      <c r="F5" s="3">
+        <v>2.81E-2</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
       </c>
       <c r="H5" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I5" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1">
-        <v>6.4299999999999996E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1579,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D6" s="2" t="b">
         <v>1</v>
@@ -1588,22 +1686,25 @@
         <v>1000</v>
       </c>
       <c r="F6" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G6" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H6" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I6" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I6" t="b">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -1611,7 +1712,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1620,22 +1721,25 @@
         <v>1000</v>
       </c>
       <c r="F7" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G7" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H7" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I7" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1747,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -1652,22 +1756,25 @@
         <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G8" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H8" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I8" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1">
-        <v>6.4299999999999996E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1675,7 +1782,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="11">
-        <v>9.45E+19</v>
+        <v>7.86E+19</v>
       </c>
       <c r="D9" s="2" t="b">
         <v>1</v>
@@ -1684,19 +1791,302 @@
         <v>1000</v>
       </c>
       <c r="F9" s="3">
-        <v>3.0099999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G9" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H9" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I9" s="4">
         <v>5100000000000</v>
       </c>
-      <c r="I9" t="b">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1">
-        <v>6.4299999999999996E-2</v>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C10" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I10" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F11" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I11" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C12" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I12" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C13" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I13" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C14" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F14" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I14" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C15" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F15" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I15" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I16" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" s="1">
+        <v>7.2300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11">
+        <v>7.86E+19</v>
+      </c>
+      <c r="D17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F17" s="3">
+        <v>2.81E-2</v>
+      </c>
+      <c r="G17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="4">
+        <v>150000</v>
+      </c>
+      <c r="I17" s="4">
+        <v>5100000000000</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" s="1">
+        <v>7.2300000000000003E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>